<commit_message>
Formaterung & FN Korrektur
</commit_message>
<xml_diff>
--- a/assets/excel/2026_5-1-2.xlsx
+++ b/assets/excel/2026_5-1-2.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDDAC2CE-14AE-452E-A80B-3956D7DA8F32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{784EAAA1-CD3C-44F2-B823-7F0E24E73403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{4424B46B-A95E-48DA-B113-8E8F86BF46C8}"/>
+    <workbookView xWindow="20052" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4424B46B-A95E-48DA-B113-8E8F86BF46C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -140,9 +140,6 @@
     <t xml:space="preserve">Frauen </t>
   </si>
   <si>
-    <t xml:space="preserve">1) Hochrechnung anhand der Bevölkerungsfortschreibung auf Basis des Zensus 2011. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe. Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren. </t>
-  </si>
-  <si>
     <t>2) Bezogen auf die Bevölkerung im Erwerbsalter (15 bis unter 65 Jahre).</t>
   </si>
   <si>
@@ -171,6 +168,9 @@
   </si>
   <si>
     <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,                                     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren. </t>
   </si>
 </sst>
 </file>
@@ -442,11 +442,11 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -455,6 +455,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -470,22 +485,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -508,9 +508,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -548,7 +548,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -654,7 +654,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -796,7 +796,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -823,22 +823,22 @@
   <sheetData>
     <row r="1" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
       <c r="M3" s="8"/>
     </row>
     <row r="4" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -858,36 +858,36 @@
       <c r="I5" s="10"/>
     </row>
     <row r="6" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="35" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24" t="s">
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="J6" s="24"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="24"/>
-      <c r="M6" s="24"/>
-      <c r="N6" s="24" t="s">
+      <c r="J6" s="33"/>
+      <c r="K6" s="33"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="O6" s="24"/>
-      <c r="P6" s="24"/>
-      <c r="Q6" s="24"/>
-      <c r="R6" s="25"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="33"/>
+      <c r="R6" s="38"/>
     </row>
     <row r="7" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="31"/>
+      <c r="B7" s="36"/>
       <c r="C7" s="27"/>
       <c r="D7" s="26" t="s">
         <v>7</v>
@@ -915,51 +915,51 @@
       </c>
       <c r="P7" s="26"/>
       <c r="Q7" s="26"/>
-      <c r="R7" s="35"/>
+      <c r="R7" s="29"/>
     </row>
     <row r="8" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="31"/>
+      <c r="B8" s="36"/>
       <c r="C8" s="27"/>
       <c r="D8" s="27"/>
-      <c r="E8" s="36" t="s">
+      <c r="E8" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="G8" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="24"/>
+      <c r="H8" s="33"/>
       <c r="I8" s="27"/>
-      <c r="J8" s="36" t="s">
+      <c r="J8" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="K8" s="37" t="s">
+      <c r="K8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="24" t="s">
+      <c r="L8" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="M8" s="24"/>
+      <c r="M8" s="33"/>
       <c r="N8" s="27"/>
-      <c r="O8" s="36" t="s">
+      <c r="O8" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="P8" s="37" t="s">
+      <c r="P8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="Q8" s="24" t="s">
+      <c r="Q8" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="R8" s="25"/>
+      <c r="R8" s="38"/>
     </row>
     <row r="9" spans="2:19" s="5" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="31"/>
+      <c r="B9" s="36"/>
       <c r="C9" s="27"/>
       <c r="D9" s="28"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="38"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="32"/>
       <c r="G9" s="11" t="s">
         <v>12</v>
       </c>
@@ -967,8 +967,8 @@
         <v>13</v>
       </c>
       <c r="I9" s="28"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="38"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="32"/>
       <c r="L9" s="11" t="s">
         <v>12</v>
       </c>
@@ -976,8 +976,8 @@
         <v>13</v>
       </c>
       <c r="N9" s="28"/>
-      <c r="O9" s="36"/>
-      <c r="P9" s="38"/>
+      <c r="O9" s="30"/>
+      <c r="P9" s="32"/>
       <c r="Q9" s="11" t="s">
         <v>12</v>
       </c>
@@ -986,25 +986,25 @@
       </c>
     </row>
     <row r="10" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="32"/>
+      <c r="B10" s="37"/>
       <c r="C10" s="28"/>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
-      <c r="N10" s="24"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="24"/>
-      <c r="R10" s="25"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="33"/>
+      <c r="N10" s="33"/>
+      <c r="O10" s="33"/>
+      <c r="P10" s="33"/>
+      <c r="Q10" s="33"/>
+      <c r="R10" s="38"/>
     </row>
     <row r="11" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="13">
@@ -3516,22 +3516,22 @@
       <c r="N58" s="17"/>
     </row>
     <row r="59" spans="2:19" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="C59" s="33"/>
-      <c r="D59" s="33"/>
-      <c r="E59" s="33"/>
-      <c r="F59" s="33"/>
-      <c r="G59" s="33"/>
-      <c r="H59" s="33"/>
-      <c r="I59" s="33"/>
-      <c r="J59" s="33"/>
-      <c r="K59" s="33"/>
+      <c r="B59" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C59" s="24"/>
+      <c r="D59" s="24"/>
+      <c r="E59" s="24"/>
+      <c r="F59" s="24"/>
+      <c r="G59" s="24"/>
+      <c r="H59" s="24"/>
+      <c r="I59" s="24"/>
+      <c r="J59" s="24"/>
+      <c r="K59" s="24"/>
     </row>
     <row r="60" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B60" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C60" s="16"/>
       <c r="D60" s="16"/>
@@ -3545,36 +3545,36 @@
       <c r="N60" s="17"/>
     </row>
     <row r="61" spans="2:19" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="34" t="s">
+      <c r="B61" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C61" s="25"/>
+      <c r="D61" s="25"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="25"/>
+      <c r="G61" s="25"/>
+      <c r="H61" s="25"/>
+      <c r="I61" s="25"/>
+      <c r="J61" s="25"/>
+      <c r="K61" s="25"/>
+    </row>
+    <row r="62" spans="2:19" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C61" s="34"/>
-      <c r="D61" s="34"/>
-      <c r="E61" s="34"/>
-      <c r="F61" s="34"/>
-      <c r="G61" s="34"/>
-      <c r="H61" s="34"/>
-      <c r="I61" s="34"/>
-      <c r="J61" s="34"/>
-      <c r="K61" s="34"/>
-    </row>
-    <row r="62" spans="2:19" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="C62" s="34"/>
-      <c r="D62" s="34"/>
-      <c r="E62" s="34"/>
-      <c r="F62" s="34"/>
-      <c r="G62" s="34"/>
-      <c r="H62" s="34"/>
-      <c r="I62" s="34"/>
-      <c r="J62" s="34"/>
-      <c r="K62" s="34"/>
+      <c r="C62" s="25"/>
+      <c r="D62" s="25"/>
+      <c r="E62" s="25"/>
+      <c r="F62" s="25"/>
+      <c r="G62" s="25"/>
+      <c r="H62" s="25"/>
+      <c r="I62" s="25"/>
+      <c r="J62" s="25"/>
+      <c r="K62" s="25"/>
     </row>
     <row r="63" spans="2:19" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C63" s="20"/>
       <c r="D63" s="20"/>
@@ -3600,7 +3600,7 @@
     </row>
     <row r="65" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C65" s="22"/>
       <c r="D65" s="22"/>
@@ -3615,7 +3615,7 @@
     <row r="66" spans="2:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C67" s="22"/>
       <c r="D67" s="22"/>
@@ -3629,7 +3629,7 @@
     </row>
     <row r="68" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C68" s="22"/>
       <c r="D68" s="22"/>
@@ -3643,7 +3643,7 @@
     </row>
     <row r="69" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C69" s="22"/>
       <c r="D69" s="22"/>
@@ -3657,7 +3657,7 @@
     </row>
     <row r="70" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C70" s="22"/>
       <c r="D70" s="22"/>
@@ -3671,6 +3671,18 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="C6:C10"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="I6:M6"/>
+    <mergeCell ref="D10:R10"/>
+    <mergeCell ref="N6:R6"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="Q8:R8"/>
     <mergeCell ref="B59:K59"/>
     <mergeCell ref="B61:K61"/>
     <mergeCell ref="B62:K62"/>
@@ -3684,18 +3696,6 @@
     <mergeCell ref="L8:M8"/>
     <mergeCell ref="O8:O9"/>
     <mergeCell ref="P8:P9"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="C6:C10"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="I6:M6"/>
-    <mergeCell ref="D10:R10"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="Q8:R8"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B70" r:id="rId1" xr:uid="{3ECA3C8E-D001-4E48-A48D-3E856F57D422}"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 9346d48b9247bca4e516cd6ea80e1e099a799b1e 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_5-1-2.xlsx
+++ b/assets/excel/2026_5-1-2.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDDAC2CE-14AE-452E-A80B-3956D7DA8F32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{784EAAA1-CD3C-44F2-B823-7F0E24E73403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{4424B46B-A95E-48DA-B113-8E8F86BF46C8}"/>
+    <workbookView xWindow="20052" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4424B46B-A95E-48DA-B113-8E8F86BF46C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -140,9 +140,6 @@
     <t xml:space="preserve">Frauen </t>
   </si>
   <si>
-    <t xml:space="preserve">1) Hochrechnung anhand der Bevölkerungsfortschreibung auf Basis des Zensus 2011. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe. Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren. </t>
-  </si>
-  <si>
     <t>2) Bezogen auf die Bevölkerung im Erwerbsalter (15 bis unter 65 Jahre).</t>
   </si>
   <si>
@@ -171,6 +168,9 @@
   </si>
   <si>
     <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,                                     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren. </t>
   </si>
 </sst>
 </file>
@@ -442,11 +442,11 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -455,6 +455,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -470,22 +485,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -508,9 +508,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -548,7 +548,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -654,7 +654,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -796,7 +796,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -823,22 +823,22 @@
   <sheetData>
     <row r="1" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
       <c r="M3" s="8"/>
     </row>
     <row r="4" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -858,36 +858,36 @@
       <c r="I5" s="10"/>
     </row>
     <row r="6" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="35" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24" t="s">
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="J6" s="24"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="24"/>
-      <c r="M6" s="24"/>
-      <c r="N6" s="24" t="s">
+      <c r="J6" s="33"/>
+      <c r="K6" s="33"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="O6" s="24"/>
-      <c r="P6" s="24"/>
-      <c r="Q6" s="24"/>
-      <c r="R6" s="25"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="33"/>
+      <c r="R6" s="38"/>
     </row>
     <row r="7" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="31"/>
+      <c r="B7" s="36"/>
       <c r="C7" s="27"/>
       <c r="D7" s="26" t="s">
         <v>7</v>
@@ -915,51 +915,51 @@
       </c>
       <c r="P7" s="26"/>
       <c r="Q7" s="26"/>
-      <c r="R7" s="35"/>
+      <c r="R7" s="29"/>
     </row>
     <row r="8" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="31"/>
+      <c r="B8" s="36"/>
       <c r="C8" s="27"/>
       <c r="D8" s="27"/>
-      <c r="E8" s="36" t="s">
+      <c r="E8" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="G8" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="24"/>
+      <c r="H8" s="33"/>
       <c r="I8" s="27"/>
-      <c r="J8" s="36" t="s">
+      <c r="J8" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="K8" s="37" t="s">
+      <c r="K8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="24" t="s">
+      <c r="L8" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="M8" s="24"/>
+      <c r="M8" s="33"/>
       <c r="N8" s="27"/>
-      <c r="O8" s="36" t="s">
+      <c r="O8" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="P8" s="37" t="s">
+      <c r="P8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="Q8" s="24" t="s">
+      <c r="Q8" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="R8" s="25"/>
+      <c r="R8" s="38"/>
     </row>
     <row r="9" spans="2:19" s="5" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="31"/>
+      <c r="B9" s="36"/>
       <c r="C9" s="27"/>
       <c r="D9" s="28"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="38"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="32"/>
       <c r="G9" s="11" t="s">
         <v>12</v>
       </c>
@@ -967,8 +967,8 @@
         <v>13</v>
       </c>
       <c r="I9" s="28"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="38"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="32"/>
       <c r="L9" s="11" t="s">
         <v>12</v>
       </c>
@@ -976,8 +976,8 @@
         <v>13</v>
       </c>
       <c r="N9" s="28"/>
-      <c r="O9" s="36"/>
-      <c r="P9" s="38"/>
+      <c r="O9" s="30"/>
+      <c r="P9" s="32"/>
       <c r="Q9" s="11" t="s">
         <v>12</v>
       </c>
@@ -986,25 +986,25 @@
       </c>
     </row>
     <row r="10" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="32"/>
+      <c r="B10" s="37"/>
       <c r="C10" s="28"/>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
-      <c r="N10" s="24"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="24"/>
-      <c r="R10" s="25"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="33"/>
+      <c r="N10" s="33"/>
+      <c r="O10" s="33"/>
+      <c r="P10" s="33"/>
+      <c r="Q10" s="33"/>
+      <c r="R10" s="38"/>
     </row>
     <row r="11" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="13">
@@ -3516,22 +3516,22 @@
       <c r="N58" s="17"/>
     </row>
     <row r="59" spans="2:19" s="18" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="C59" s="33"/>
-      <c r="D59" s="33"/>
-      <c r="E59" s="33"/>
-      <c r="F59" s="33"/>
-      <c r="G59" s="33"/>
-      <c r="H59" s="33"/>
-      <c r="I59" s="33"/>
-      <c r="J59" s="33"/>
-      <c r="K59" s="33"/>
+      <c r="B59" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C59" s="24"/>
+      <c r="D59" s="24"/>
+      <c r="E59" s="24"/>
+      <c r="F59" s="24"/>
+      <c r="G59" s="24"/>
+      <c r="H59" s="24"/>
+      <c r="I59" s="24"/>
+      <c r="J59" s="24"/>
+      <c r="K59" s="24"/>
     </row>
     <row r="60" spans="2:19" s="5" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B60" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C60" s="16"/>
       <c r="D60" s="16"/>
@@ -3545,36 +3545,36 @@
       <c r="N60" s="17"/>
     </row>
     <row r="61" spans="2:19" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="34" t="s">
+      <c r="B61" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C61" s="25"/>
+      <c r="D61" s="25"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="25"/>
+      <c r="G61" s="25"/>
+      <c r="H61" s="25"/>
+      <c r="I61" s="25"/>
+      <c r="J61" s="25"/>
+      <c r="K61" s="25"/>
+    </row>
+    <row r="62" spans="2:19" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C61" s="34"/>
-      <c r="D61" s="34"/>
-      <c r="E61" s="34"/>
-      <c r="F61" s="34"/>
-      <c r="G61" s="34"/>
-      <c r="H61" s="34"/>
-      <c r="I61" s="34"/>
-      <c r="J61" s="34"/>
-      <c r="K61" s="34"/>
-    </row>
-    <row r="62" spans="2:19" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="C62" s="34"/>
-      <c r="D62" s="34"/>
-      <c r="E62" s="34"/>
-      <c r="F62" s="34"/>
-      <c r="G62" s="34"/>
-      <c r="H62" s="34"/>
-      <c r="I62" s="34"/>
-      <c r="J62" s="34"/>
-      <c r="K62" s="34"/>
+      <c r="C62" s="25"/>
+      <c r="D62" s="25"/>
+      <c r="E62" s="25"/>
+      <c r="F62" s="25"/>
+      <c r="G62" s="25"/>
+      <c r="H62" s="25"/>
+      <c r="I62" s="25"/>
+      <c r="J62" s="25"/>
+      <c r="K62" s="25"/>
     </row>
     <row r="63" spans="2:19" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C63" s="20"/>
       <c r="D63" s="20"/>
@@ -3600,7 +3600,7 @@
     </row>
     <row r="65" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C65" s="22"/>
       <c r="D65" s="22"/>
@@ -3615,7 +3615,7 @@
     <row r="66" spans="2:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C67" s="22"/>
       <c r="D67" s="22"/>
@@ -3629,7 +3629,7 @@
     </row>
     <row r="68" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C68" s="22"/>
       <c r="D68" s="22"/>
@@ -3643,7 +3643,7 @@
     </row>
     <row r="69" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C69" s="22"/>
       <c r="D69" s="22"/>
@@ -3657,7 +3657,7 @@
     </row>
     <row r="70" spans="2:11" s="18" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C70" s="22"/>
       <c r="D70" s="22"/>
@@ -3671,6 +3671,18 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="C6:C10"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="I6:M6"/>
+    <mergeCell ref="D10:R10"/>
+    <mergeCell ref="N6:R6"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="Q8:R8"/>
     <mergeCell ref="B59:K59"/>
     <mergeCell ref="B61:K61"/>
     <mergeCell ref="B62:K62"/>
@@ -3684,18 +3696,6 @@
     <mergeCell ref="L8:M8"/>
     <mergeCell ref="O8:O9"/>
     <mergeCell ref="P8:P9"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="C6:C10"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="I6:M6"/>
-    <mergeCell ref="D10:R10"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="Q8:R8"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B70" r:id="rId1" xr:uid="{3ECA3C8E-D001-4E48-A48D-3E856F57D422}"/>

</xml_diff>